<commit_message>
Dashboard map and query table for crops done
</commit_message>
<xml_diff>
--- a/master_db_agrobotanix.xlsx
+++ b/master_db_agrobotanix.xlsx
@@ -33,11 +33,11 @@
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
   <authors>
-    <author>tc={24e64f24-e499-4e98-8f11-07b15e55f20e}</author>
-    <author>tc={4252ba9d-a9fb-4550-93de-5a93ee78a1a1}</author>
+    <author>tc={7345dc5e-8c95-4b84-bfb7-b2e1a578187d}</author>
+    <author>tc={acbc27b3-ed92-47d7-af03-78528d0523f4}</author>
   </authors>
   <commentList>
-    <comment authorId="0" xr:uid="{24e64f24-e499-4e98-8f11-07b15e55f20e}" ref="F1">
+    <comment authorId="0" xr:uid="{7345dc5e-8c95-4b84-bfb7-b2e1a578187d}" ref="F1">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -46,7 +46,7 @@
 </t>
       </text>
     </comment>
-    <comment authorId="1" xr:uid="{4252ba9d-a9fb-4550-93de-5a93ee78a1a1}" ref="G1">
+    <comment authorId="1" xr:uid="{acbc27b3-ed92-47d7-af03-78528d0523f4}" ref="G1">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -62,10 +62,10 @@
 <file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
   <authors>
-    <author>tc={c5d9bbb9-aaa1-4bb4-a0b3-3e8a29b7fb77}</author>
+    <author>tc={a0635af6-157a-492d-8e18-44acef0d413d}</author>
   </authors>
   <commentList>
-    <comment authorId="0" xr:uid="{c5d9bbb9-aaa1-4bb4-a0b3-3e8a29b7fb77}" ref="B1">
+    <comment authorId="0" xr:uid="{a0635af6-157a-492d-8e18-44acef0d413d}" ref="B1">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -79,7 +79,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4674" uniqueCount="993">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4676" uniqueCount="993">
   <si>
     <t>cultivo</t>
   </si>
@@ -3549,7 +3549,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <x18tc:person displayName="Jesus Alejandro Barquin Ortiz" id="{31000369-0178-4af1-a428-cc62758a712b}" providerId="google-sheets"/>
+  <x18tc:person displayName="Jesus Alejandro Barquin Ortiz" id="{b51b13fa-9796-44b0-aca7-6602b4a2fa1f}" providerId="google-sheets"/>
 </x18tc:personList>
 </file>
 
@@ -3823,10 +3823,10 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <x18tc:threadedComment ref="G1" dT="2026-03-04T21:20:20.00" personId="{31000369-0178-4af1-a428-cc62758a712b}" id="{4252ba9d-a9fb-4550-93de-5a93ee78a1a1}" done="0">
+  <x18tc:threadedComment ref="G1" dT="2026-03-04T21:20:20.00" personId="{b51b13fa-9796-44b0-aca7-6602b4a2fa1f}" id="{acbc27b3-ed92-47d7-af03-78528d0523f4}" done="0">
     <x18tc:text xml:space="preserve">estas las obtuve del csv del cierre agricola del siap en 2024</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="F1" dT="2026-03-04T21:20:31.00" personId="{31000369-0178-4af1-a428-cc62758a712b}" id="{24e64f24-e499-4e98-8f11-07b15e55f20e}" done="0">
+  <x18tc:threadedComment ref="F1" dT="2026-03-04T21:20:31.00" personId="{b51b13fa-9796-44b0-aca7-6602b4a2fa1f}" id="{7345dc5e-8c95-4b84-bfb7-b2e1a578187d}" done="0">
     <x18tc:text xml:space="preserve">estas las obtuve del csv del cierre agricola del siap en 2024</x18tc:text>
   </x18tc:threadedComment>
 </x18tc:ThreadedComments>
@@ -3834,7 +3834,7 @@
 
 <file path=xl/threadedComments/threadedComment2.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <x18tc:threadedComment ref="B1" dT="2026-03-03T21:20:58.00" personId="{31000369-0178-4af1-a428-cc62758a712b}" id="{c5d9bbb9-aaa1-4bb4-a0b3-3e8a29b7fb77}" done="0">
+  <x18tc:threadedComment ref="B1" dT="2026-03-03T21:20:58.00" personId="{b51b13fa-9796-44b0-aca7-6602b4a2fa1f}" id="{a0635af6-157a-492d-8e18-44acef0d413d}" done="0">
     <x18tc:text xml:space="preserve">Este se puede obtener del documento de panorama agrolimentario</x18tc:text>
   </x18tc:threadedComment>
 </x18tc:ThreadedComments>
@@ -20733,7 +20733,6 @@
         <v>0.78</v>
       </c>
       <c r="E10" s="40"/>
-      <c r="F10" s="37"/>
       <c r="G10" s="37"/>
     </row>
     <row r="11" ht="22.5" customHeight="1">
@@ -20743,7 +20742,6 @@
       <c r="B11" s="36">
         <v>0.6</v>
       </c>
-      <c r="F11" s="40"/>
       <c r="G11" s="40"/>
     </row>
     <row r="12" ht="22.5" customHeight="1">
@@ -20789,9 +20787,17 @@
       </c>
     </row>
     <row r="17" ht="22.5" customHeight="1">
-      <c r="B17" s="38"/>
+      <c r="A17" s="24" t="s">
+        <v>773</v>
+      </c>
+      <c r="B17" s="36">
+        <v>0.92</v>
+      </c>
     </row>
     <row r="18" ht="22.5" customHeight="1">
+      <c r="A18" s="27" t="s">
+        <v>794</v>
+      </c>
       <c r="B18" s="38"/>
     </row>
     <row r="19" ht="22.5" customHeight="1">

</xml_diff>